<commit_message>
feature : ItemActor / C_InteractionReceive 구현
AA_Character_Player : Item 확인을 위한 Test코드 추가
UC_InteractionReceive : Interactor 받는 액터의 컴포넌트
                               Collision을 Bind 해주고 BOOL 설정에 의해 자/수동으로 CollisionEvent 발생
UC_InteractionReceive_Item :
                               E_BeginEvent_Detect_Implementation 은 Initiator와 충돌이 있으면 발생
                               E_EndEvent_Detect_Implementation 은 충돌이 끝나면 발생
                               E_BeginEvent_Interaction_Implementation은 자동: 충돌하면 발생 / 수동 : Initiator가 호출하면 발생
                               E_EndEvent_Interaction_Implementation은 자동: 충돌하면 발생 / 수동 : Initiator가 호출하면 발생
Item.h S_Item : Item에 필요한 Enum class 와 Struct 구현
</commit_message>
<xml_diff>
--- a/코드 파일 기술서.xlsx
+++ b/코드 파일 기술서.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\source\repos\Unreal\UE5\TopDownPortfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C12C9F-0CE6-4F22-8DD4-A5598583E5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62A5BF95-78B4-4B21-89AD-EC09535141E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{D21DC332-3B34-4EF0-AFA4-A1E5433A082F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="6" xr2:uid="{D21DC332-3B34-4EF0-AFA4-A1E5433A082F}"/>
   </bookViews>
   <sheets>
     <sheet name="코드 작성 양식" sheetId="2" r:id="rId1"/>
@@ -19,8 +19,9 @@
     <sheet name="MontagMGR" sheetId="1" r:id="rId4"/>
     <sheet name="AIActionMGR" sheetId="7" r:id="rId5"/>
     <sheet name="StateMGR" sheetId="8" r:id="rId6"/>
-    <sheet name="SkillMGR" sheetId="5" r:id="rId7"/>
-    <sheet name="TargetMGR" sheetId="3" r:id="rId8"/>
+    <sheet name="A_InteractionActor" sheetId="9" r:id="rId7"/>
+    <sheet name="SkillMGR" sheetId="5" r:id="rId8"/>
+    <sheet name="TargetMGR" sheetId="3" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="111">
   <si>
     <t>개요</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -76,10 +77,6 @@
   </si>
   <si>
     <t xml:space="preserve"> 작성 이유</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> 클래스의 목적</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -524,12 +521,44 @@
     <t>캐릭터의 StateType이나 CharacterType 처럼 캐릭터의 상태나 관계 Hit 여부 등을 통합 관리한다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>A_InteractionActor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CollisionOverlap을 통해 Player 혹은 몬스터 등과 상호 작용 하는 Actor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>계획</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> 클래스의 설계 꼐획</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>InteractionEvent와 DetectedEvent는 상속으로 재정의</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>해당 액터의 Collision충돌시 DetectedEvent 자동 실행 (토글 가능)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(충돌될 객체의 Collision을 여러 개 두개 할지 Enum으로 구별할 지 고민중 InteractionID가 있어서 충돌이 겹쳐도 가능하게)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>해당 액터랑 충돌한 Actor의 컴포넌트가 알아서 InteractionEvent 메소드 실행 (토글 가능)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -597,6 +626,14 @@
     </font>
     <font>
       <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="함초롬돋움"/>
+      <family val="1"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <strike/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="함초롬돋움"/>
@@ -1027,7 +1064,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1073,13 +1110,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1109,10 +1152,19 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1133,19 +1185,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1490,56 +1536,56 @@
   <sheetData>
     <row r="1" spans="2:18" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:18" ht="17.25" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
       <c r="Q2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="R2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="2:18">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
       <c r="Q3" s="1"/>
       <c r="R3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="2:18">
       <c r="B4" s="2"/>
-      <c r="C4" s="15"/>
+      <c r="C4" s="18"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -1555,10 +1601,10 @@
     </row>
     <row r="5" spans="2:18">
       <c r="B5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>9</v>
+        <v>105</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>106</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -1575,7 +1621,7 @@
     </row>
     <row r="6" spans="2:18">
       <c r="B6" s="6"/>
-      <c r="C6" s="15"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -1591,19 +1637,19 @@
     </row>
     <row r="7" spans="2:18">
       <c r="B7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="18" t="s">
         <v>16</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>17</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="28" t="s">
-        <v>38</v>
+      <c r="I7" s="19"/>
+      <c r="J7" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="K7" s="16"/>
       <c r="L7" s="16"/>
@@ -1613,14 +1659,14 @@
     </row>
     <row r="8" spans="2:18">
       <c r="B8" s="6"/>
-      <c r="C8" s="15"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="28"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="15"/>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
@@ -1629,10 +1675,10 @@
     </row>
     <row r="9" spans="2:18">
       <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -1649,7 +1695,7 @@
     </row>
     <row r="10" spans="2:18">
       <c r="B10" s="6"/>
-      <c r="C10" s="15"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -1667,13 +1713,13 @@
       <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="15" t="s">
         <v>43</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28" t="s">
-        <v>44</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
@@ -1687,10 +1733,10 @@
     </row>
     <row r="12" spans="2:18">
       <c r="B12" s="6"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -1705,13 +1751,13 @@
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>45</v>
+      <c r="C13" s="18" t="s">
+        <v>44</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28" t="s">
-        <v>44</v>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15" t="s">
+        <v>43</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
@@ -1727,10 +1773,10 @@
       <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="15"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -1743,10 +1789,10 @@
     </row>
     <row r="15" spans="2:18" ht="17.25" thickBot="1">
       <c r="B15" s="4"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="18"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -1759,27 +1805,27 @@
     </row>
     <row r="16" spans="2:18">
       <c r="B16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="21"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="21"/>
+      <c r="N16" s="21"/>
+      <c r="O16" s="22"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="6"/>
-      <c r="C17" s="15"/>
+      <c r="C17" s="18"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
@@ -1795,32 +1841,24 @@
     </row>
     <row r="18" spans="2:15" ht="17.25" thickBot="1">
       <c r="B18" s="10"/>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="23"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
+      <c r="O18" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="F11:O11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:O12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
     <mergeCell ref="C17:O17"/>
     <mergeCell ref="C16:O16"/>
     <mergeCell ref="C18:O18"/>
@@ -1837,6 +1875,14 @@
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
     <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:O11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="F12:O12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1850,46 +1896,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="C3" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="2:15" ht="15" customHeight="1">
       <c r="B4" s="2"/>
-      <c r="C4" s="15"/>
+      <c r="C4" s="18"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -1907,8 +1953,8 @@
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>48</v>
+      <c r="C5" s="18" t="s">
+        <v>47</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -1925,8 +1971,8 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="6"/>
-      <c r="C6" s="15" t="s">
-        <v>49</v>
+      <c r="C6" s="18" t="s">
+        <v>48</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -1943,7 +1989,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="15"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -1959,17 +2005,17 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="15"/>
+        <v>15</v>
+      </c>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="28" t="s">
-        <v>38</v>
+      <c r="I8" s="19"/>
+      <c r="J8" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
@@ -1979,14 +2025,14 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="15"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="28"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="15"/>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
@@ -1995,10 +2041,10 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>51</v>
+        <v>18</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>50</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
@@ -2015,7 +2061,7 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="15"/>
+      <c r="C11" s="18"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -2033,13 +2079,13 @@
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>50</v>
+      <c r="C12" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="D12" s="16"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28" t="s">
-        <v>44</v>
+      <c r="E12" s="19"/>
+      <c r="F12" s="15" t="s">
+        <v>43</v>
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
@@ -2053,10 +2099,10 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="15"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
@@ -2069,10 +2115,10 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="15"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -2087,13 +2133,13 @@
       <c r="B15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="15" t="s">
-        <v>45</v>
+      <c r="C15" s="18" t="s">
+        <v>44</v>
       </c>
       <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28" t="s">
-        <v>44</v>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15" t="s">
+        <v>43</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -2109,10 +2155,10 @@
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="15"/>
+      <c r="C16" s="18"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="28"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -2125,10 +2171,10 @@
     </row>
     <row r="17" spans="2:15" ht="17.25" thickBot="1">
       <c r="B17" s="4"/>
-      <c r="C17" s="15"/>
+      <c r="C17" s="18"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -2141,27 +2187,27 @@
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="22"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="6"/>
-      <c r="C19" s="15"/>
+      <c r="C19" s="18"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
@@ -2177,29 +2223,32 @@
     </row>
     <row r="20" spans="2:15" ht="17.25" thickBot="1">
       <c r="B20" s="10"/>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C18:O18"/>
-    <mergeCell ref="C19:O19"/>
-    <mergeCell ref="C20:O20"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F16:O16"/>
     <mergeCell ref="C9:I9"/>
@@ -2214,14 +2263,11 @@
     <mergeCell ref="F14:O14"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="F15:O15"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:O17"/>
+    <mergeCell ref="C18:O18"/>
+    <mergeCell ref="C19:O19"/>
+    <mergeCell ref="C20:O20"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2235,47 +2281,47 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="C3" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="15" t="s">
-        <v>86</v>
+      <c r="C4" s="18" t="s">
+        <v>85</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -2292,7 +2338,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="15"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -2310,8 +2356,8 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>60</v>
+      <c r="C6" s="18" t="s">
+        <v>59</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -2328,8 +2374,8 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="15" t="s">
-        <v>83</v>
+      <c r="C7" s="18" t="s">
+        <v>82</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -2346,7 +2392,7 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="15"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -2362,19 +2408,19 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>16</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>17</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="28" t="s">
-        <v>38</v>
+      <c r="I9" s="19"/>
+      <c r="J9" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
@@ -2384,14 +2430,14 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="15"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="28"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="15"/>
       <c r="K10" s="16"/>
       <c r="L10" s="16"/>
       <c r="M10" s="16"/>
@@ -2400,10 +2446,10 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>61</v>
+        <v>18</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>60</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
@@ -2420,7 +2466,7 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
@@ -2438,13 +2484,13 @@
       <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>80</v>
+      <c r="C13" s="18" t="s">
+        <v>79</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28" t="s">
-        <v>72</v>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15" t="s">
+        <v>71</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
@@ -2458,10 +2504,10 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="15"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -2476,13 +2522,13 @@
       <c r="B15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15" t="s">
         <v>81</v>
-      </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28" t="s">
-        <v>82</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -2498,10 +2544,10 @@
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="15"/>
+      <c r="C16" s="18"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="28"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -2514,10 +2560,10 @@
     </row>
     <row r="17" spans="2:15" ht="17.25" thickBot="1">
       <c r="B17" s="4"/>
-      <c r="C17" s="15"/>
+      <c r="C17" s="18"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -2530,25 +2576,25 @@
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="20"/>
+        <v>35</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="22"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="6"/>
-      <c r="C19" s="15"/>
+      <c r="C19" s="18"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
@@ -2564,64 +2610,64 @@
     </row>
     <row r="20" spans="2:15" ht="17.25" thickBot="1">
       <c r="B20" s="10"/>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="25"/>
     </row>
     <row r="22" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="23" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B23" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="25"/>
-      <c r="N23" s="25"/>
-      <c r="O23" s="26"/>
+      <c r="B23" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="28"/>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="19"/>
-      <c r="O24" s="20"/>
+      <c r="C24" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="21"/>
+      <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="22"/>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2"/>
-      <c r="C25" s="15"/>
+      <c r="C25" s="18"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
@@ -2637,7 +2683,7 @@
     </row>
     <row r="26" spans="2:15">
       <c r="B26" s="2"/>
-      <c r="C26" s="15"/>
+      <c r="C26" s="18"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
@@ -2655,7 +2701,7 @@
       <c r="B27" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C27" s="15"/>
+      <c r="C27" s="18"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
@@ -2671,7 +2717,7 @@
     </row>
     <row r="28" spans="2:15">
       <c r="B28" s="6"/>
-      <c r="C28" s="15"/>
+      <c r="C28" s="18"/>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
@@ -2687,18 +2733,18 @@
     </row>
     <row r="29" spans="2:15">
       <c r="B29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>78</v>
+        <v>15</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>77</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
       <c r="F29" s="16"/>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="28"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="15"/>
       <c r="K29" s="16"/>
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
@@ -2707,16 +2753,16 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="6"/>
-      <c r="C30" s="15" t="s">
-        <v>79</v>
+      <c r="C30" s="18" t="s">
+        <v>78</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="16"/>
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="28"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="15"/>
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
@@ -2725,14 +2771,14 @@
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="6"/>
-      <c r="C31" s="15"/>
+      <c r="C31" s="18"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="28"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="15"/>
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
@@ -2741,9 +2787,9 @@
     </row>
     <row r="32" spans="2:15">
       <c r="B32" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C32" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="C32" s="18"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
@@ -2759,7 +2805,7 @@
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="6"/>
-      <c r="C33" s="15"/>
+      <c r="C33" s="18"/>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
       <c r="F33" s="16"/>
@@ -2777,13 +2823,13 @@
       <c r="B34" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="15" t="s">
-        <v>73</v>
+      <c r="C34" s="18" t="s">
+        <v>72</v>
       </c>
       <c r="D34" s="16"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="28" t="s">
-        <v>75</v>
+      <c r="E34" s="19"/>
+      <c r="F34" s="15" t="s">
+        <v>74</v>
       </c>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
@@ -2797,13 +2843,13 @@
     </row>
     <row r="35" spans="2:15">
       <c r="B35" s="6"/>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="16"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="15" t="s">
         <v>73</v>
-      </c>
-      <c r="D35" s="16"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="28" t="s">
-        <v>74</v>
       </c>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
@@ -2817,13 +2863,13 @@
     </row>
     <row r="36" spans="2:15">
       <c r="B36" s="6"/>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="16"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="D36" s="16"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="28" t="s">
-        <v>77</v>
       </c>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
@@ -2837,10 +2883,10 @@
     </row>
     <row r="37" spans="2:15">
       <c r="B37" s="6"/>
-      <c r="C37" s="15"/>
+      <c r="C37" s="18"/>
       <c r="D37" s="16"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="28"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="15"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
       <c r="I37" s="16"/>
@@ -2855,13 +2901,13 @@
       <c r="B38" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="16"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="15" t="s">
         <v>84</v>
-      </c>
-      <c r="D38" s="16"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="28" t="s">
-        <v>85</v>
       </c>
       <c r="G38" s="16"/>
       <c r="H38" s="16"/>
@@ -2877,10 +2923,10 @@
       <c r="B39" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="15"/>
+      <c r="C39" s="18"/>
       <c r="D39" s="16"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="28"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="15"/>
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
@@ -2893,10 +2939,10 @@
     </row>
     <row r="40" spans="2:15" ht="17.25" thickBot="1">
       <c r="B40" s="4"/>
-      <c r="C40" s="15"/>
+      <c r="C40" s="18"/>
       <c r="D40" s="16"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="28"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="15"/>
       <c r="G40" s="16"/>
       <c r="H40" s="16"/>
       <c r="I40" s="16"/>
@@ -2909,25 +2955,25 @@
     </row>
     <row r="41" spans="2:15">
       <c r="B41" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C41" s="18"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="19"/>
-      <c r="J41" s="19"/>
-      <c r="K41" s="19"/>
-      <c r="L41" s="19"/>
-      <c r="M41" s="19"/>
-      <c r="N41" s="19"/>
-      <c r="O41" s="20"/>
+        <v>35</v>
+      </c>
+      <c r="C41" s="20"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="21"/>
+      <c r="J41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+      <c r="M41" s="21"/>
+      <c r="N41" s="21"/>
+      <c r="O41" s="22"/>
     </row>
     <row r="42" spans="2:15">
       <c r="B42" s="6"/>
-      <c r="C42" s="15"/>
+      <c r="C42" s="18"/>
       <c r="D42" s="16"/>
       <c r="E42" s="16"/>
       <c r="F42" s="16"/>
@@ -2943,37 +2989,52 @@
     </row>
     <row r="43" spans="2:15" ht="17.25" thickBot="1">
       <c r="B43" s="10"/>
-      <c r="C43" s="21" t="s">
+      <c r="C43" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D43" s="22"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
-      <c r="K43" s="22"/>
-      <c r="L43" s="22"/>
-      <c r="M43" s="22"/>
-      <c r="N43" s="22"/>
-      <c r="O43" s="23"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="24"/>
+      <c r="H43" s="24"/>
+      <c r="I43" s="24"/>
+      <c r="J43" s="24"/>
+      <c r="K43" s="24"/>
+      <c r="L43" s="24"/>
+      <c r="M43" s="24"/>
+      <c r="N43" s="24"/>
+      <c r="O43" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="57">
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C10:I10"/>
-    <mergeCell ref="J10:O10"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="J9:O9"/>
-    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:O35"/>
+    <mergeCell ref="C30:I30"/>
+    <mergeCell ref="J30:O30"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="F40:O40"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="J31:O31"/>
+    <mergeCell ref="C32:O32"/>
+    <mergeCell ref="C33:O33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="F34:O34"/>
+    <mergeCell ref="C41:O41"/>
+    <mergeCell ref="C42:O42"/>
+    <mergeCell ref="C43:O43"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="F36:O36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="F37:O37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="F38:O38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="F39:O39"/>
+    <mergeCell ref="C24:O24"/>
+    <mergeCell ref="C25:O25"/>
+    <mergeCell ref="C26:O26"/>
+    <mergeCell ref="C27:O27"/>
+    <mergeCell ref="C28:O28"/>
     <mergeCell ref="C29:I29"/>
     <mergeCell ref="J29:O29"/>
     <mergeCell ref="B23:O23"/>
@@ -2990,34 +3051,19 @@
     <mergeCell ref="C12:O12"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
-    <mergeCell ref="C24:O24"/>
-    <mergeCell ref="C25:O25"/>
-    <mergeCell ref="C26:O26"/>
-    <mergeCell ref="C27:O27"/>
-    <mergeCell ref="C28:O28"/>
-    <mergeCell ref="C41:O41"/>
-    <mergeCell ref="C42:O42"/>
-    <mergeCell ref="C43:O43"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="F36:O36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="F37:O37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="F38:O38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="F39:O39"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="F35:O35"/>
-    <mergeCell ref="C30:I30"/>
-    <mergeCell ref="J30:O30"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="F40:O40"/>
-    <mergeCell ref="C31:I31"/>
-    <mergeCell ref="J31:O31"/>
-    <mergeCell ref="C32:O32"/>
-    <mergeCell ref="C33:O33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="F34:O34"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="J9:O9"/>
+    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="J10:O10"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3035,47 +3081,47 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="37"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="30"/>
+      <c r="O3" s="31"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="5"/>
-      <c r="C4" s="15" t="s">
-        <v>32</v>
+      <c r="C4" s="18" t="s">
+        <v>31</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -3092,44 +3138,44 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="5"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="37"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="31"/>
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="38"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="39"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="33"/>
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="15" t="s">
-        <v>11</v>
+      <c r="C7" s="18" t="s">
+        <v>10</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -3146,7 +3192,7 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="15"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -3162,19 +3208,19 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>23</v>
+        <v>15</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="27"/>
+      <c r="I9" s="19"/>
       <c r="J9" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
@@ -3184,17 +3230,17 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="15" t="s">
-        <v>24</v>
+      <c r="C10" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="27"/>
+      <c r="I10" s="19"/>
       <c r="J10" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K10" s="16"/>
       <c r="L10" s="16"/>
@@ -3204,17 +3250,17 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="15" t="s">
-        <v>26</v>
+      <c r="C11" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="27"/>
+      <c r="I11" s="19"/>
       <c r="J11" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K11" s="16"/>
       <c r="L11" s="16"/>
@@ -3224,13 +3270,13 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
-      <c r="I12" s="27"/>
+      <c r="I12" s="19"/>
       <c r="J12" s="16"/>
       <c r="K12" s="16"/>
       <c r="L12" s="16"/>
@@ -3240,10 +3286,10 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>33</v>
+        <v>18</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>32</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
@@ -3260,8 +3306,8 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="15" t="s">
-        <v>31</v>
+      <c r="C14" s="18" t="s">
+        <v>30</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -3278,8 +3324,8 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="6"/>
-      <c r="C15" s="15" t="s">
-        <v>34</v>
+      <c r="C15" s="18" t="s">
+        <v>33</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
@@ -3296,7 +3342,7 @@
     </row>
     <row r="16" spans="2:15">
       <c r="B16" s="6"/>
-      <c r="C16" s="15"/>
+      <c r="C16" s="18"/>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
@@ -3315,10 +3361,10 @@
         <v>7</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
@@ -3335,10 +3381,10 @@
     <row r="18" spans="2:15">
       <c r="B18" s="6"/>
       <c r="C18" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
@@ -3355,10 +3401,10 @@
     <row r="19" spans="2:15">
       <c r="B19" s="6"/>
       <c r="C19" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>14</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
@@ -3374,7 +3420,7 @@
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="6"/>
-      <c r="D20" s="28"/>
+      <c r="D20" s="15"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
       <c r="G20" s="16"/>
@@ -3390,7 +3436,7 @@
     <row r="21" spans="2:15">
       <c r="B21" s="6"/>
       <c r="C21" s="7"/>
-      <c r="D21" s="28"/>
+      <c r="D21" s="15"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
@@ -3408,10 +3454,10 @@
         <v>4</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="28" t="s">
-        <v>35</v>
+        <v>26</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
@@ -3428,10 +3474,10 @@
     <row r="23" spans="2:15">
       <c r="B23" s="3"/>
       <c r="C23" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="28" t="s">
-        <v>30</v>
+        <v>21</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
@@ -3448,10 +3494,10 @@
     <row r="24" spans="2:15">
       <c r="B24" s="3"/>
       <c r="C24" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>29</v>
+        <v>24</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>28</v>
       </c>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
@@ -3468,10 +3514,10 @@
     <row r="25" spans="2:15">
       <c r="B25" s="3"/>
       <c r="C25" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>28</v>
+        <v>20</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>27</v>
       </c>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
@@ -3504,164 +3550,153 @@
     <row r="27" spans="2:15" ht="17.25" thickBot="1">
       <c r="B27" s="4"/>
       <c r="C27" s="8"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="23"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="O27" s="25"/>
     </row>
     <row r="28" spans="2:15">
       <c r="B28" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C28" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="33"/>
-      <c r="O28" s="34"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
+      <c r="K28" s="38"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="38"/>
+      <c r="N28" s="38"/>
+      <c r="O28" s="39"/>
     </row>
     <row r="29" spans="2:15">
       <c r="B29" s="11"/>
-      <c r="C29" s="29" t="s">
-        <v>88</v>
-      </c>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="31"/>
+      <c r="C29" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" s="35"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="35"/>
+      <c r="N29" s="35"/>
+      <c r="O29" s="36"/>
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="11"/>
-      <c r="C30" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="30"/>
-      <c r="M30" s="30"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="31"/>
+      <c r="C30" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" s="35"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="35"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="36"/>
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="11"/>
-      <c r="C31" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30"/>
-      <c r="O31" s="31"/>
+      <c r="C31" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="35"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
+      <c r="K31" s="35"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
+      <c r="O31" s="36"/>
     </row>
     <row r="32" spans="2:15">
       <c r="B32" s="11"/>
-      <c r="C32" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="30"/>
-      <c r="M32" s="30"/>
-      <c r="N32" s="30"/>
-      <c r="O32" s="31"/>
+      <c r="C32" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="35"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="35"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="35"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
+      <c r="O32" s="36"/>
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="11"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
-      <c r="N33" s="30"/>
-      <c r="O33" s="31"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="35"/>
+      <c r="E33" s="35"/>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="35"/>
+      <c r="J33" s="35"/>
+      <c r="K33" s="35"/>
+      <c r="L33" s="35"/>
+      <c r="M33" s="35"/>
+      <c r="N33" s="35"/>
+      <c r="O33" s="36"/>
     </row>
     <row r="34" spans="2:15" ht="17.25" thickBot="1">
       <c r="B34" s="10"/>
-      <c r="C34" s="21" t="s">
+      <c r="C34" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="22"/>
-      <c r="O34" s="23"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="25"/>
     </row>
     <row r="40" spans="2:15" ht="17.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C13:O13"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="D26:O26"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="D19:O19"/>
-    <mergeCell ref="D24:O24"/>
-    <mergeCell ref="D21:O21"/>
-    <mergeCell ref="D20:O20"/>
-    <mergeCell ref="C16:O16"/>
-    <mergeCell ref="D17:O17"/>
-    <mergeCell ref="D18:O18"/>
+    <mergeCell ref="C31:O31"/>
+    <mergeCell ref="C29:O29"/>
+    <mergeCell ref="C30:O30"/>
+    <mergeCell ref="C32:O32"/>
+    <mergeCell ref="C28:O28"/>
     <mergeCell ref="C34:O34"/>
     <mergeCell ref="C33:O33"/>
     <mergeCell ref="C9:I9"/>
@@ -3678,11 +3713,22 @@
     <mergeCell ref="D23:O23"/>
     <mergeCell ref="D22:O22"/>
     <mergeCell ref="D25:O25"/>
-    <mergeCell ref="C31:O31"/>
-    <mergeCell ref="C29:O29"/>
-    <mergeCell ref="C30:O30"/>
-    <mergeCell ref="C32:O32"/>
-    <mergeCell ref="C28:O28"/>
+    <mergeCell ref="D26:O26"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="D19:O19"/>
+    <mergeCell ref="D24:O24"/>
+    <mergeCell ref="D21:O21"/>
+    <mergeCell ref="D20:O20"/>
+    <mergeCell ref="C16:O16"/>
+    <mergeCell ref="D17:O17"/>
+    <mergeCell ref="D18:O18"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C13:O13"/>
+    <mergeCell ref="C6:O6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3696,47 +3742,47 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="C3" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="15" t="s">
-        <v>100</v>
+      <c r="C4" s="18" t="s">
+        <v>99</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -3753,7 +3799,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="15"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -3771,8 +3817,8 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>93</v>
+      <c r="C6" s="18" t="s">
+        <v>92</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -3789,8 +3835,8 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="15" t="s">
-        <v>94</v>
+      <c r="C7" s="18" t="s">
+        <v>93</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -3807,7 +3853,7 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="15"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -3823,7 +3869,7 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="15"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
@@ -3839,19 +3885,19 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="18" t="s">
         <v>16</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>17</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="28" t="s">
-        <v>38</v>
+      <c r="I10" s="19"/>
+      <c r="J10" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="K10" s="16"/>
       <c r="L10" s="16"/>
@@ -3861,14 +3907,14 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="15"/>
+      <c r="C11" s="18"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="28"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="15"/>
       <c r="K11" s="16"/>
       <c r="L11" s="16"/>
       <c r="M11" s="16"/>
@@ -3877,10 +3923,10 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>19</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
@@ -3897,7 +3943,7 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="15"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
@@ -3915,13 +3961,13 @@
       <c r="B14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>95</v>
+      <c r="C14" s="18" t="s">
+        <v>94</v>
       </c>
       <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28" t="s">
-        <v>44</v>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15" t="s">
+        <v>43</v>
       </c>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
@@ -3935,10 +3981,10 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="6"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="18"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -3953,13 +3999,13 @@
       <c r="B16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="15" t="s">
-        <v>99</v>
+      <c r="C16" s="18" t="s">
+        <v>98</v>
       </c>
       <c r="D16" s="16"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="28" t="s">
-        <v>97</v>
+      <c r="E16" s="19"/>
+      <c r="F16" s="15" t="s">
+        <v>96</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -3975,13 +4021,13 @@
       <c r="B17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="15" t="s">
-        <v>96</v>
+      <c r="C17" s="18" t="s">
+        <v>95</v>
       </c>
       <c r="D17" s="16"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28" t="s">
-        <v>98</v>
+      <c r="E17" s="19"/>
+      <c r="F17" s="15" t="s">
+        <v>97</v>
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
@@ -3995,10 +4041,10 @@
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="3"/>
-      <c r="C18" s="15"/>
+      <c r="C18" s="18"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="28"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="15"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
@@ -4011,10 +4057,10 @@
     </row>
     <row r="19" spans="2:15" ht="17.25" thickBot="1">
       <c r="B19" s="4"/>
-      <c r="C19" s="15"/>
+      <c r="C19" s="18"/>
       <c r="D19" s="16"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="15"/>
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
@@ -4027,27 +4073,27 @@
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="22"/>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="6"/>
-      <c r="C21" s="15"/>
+      <c r="C21" s="18"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
@@ -4063,24 +4109,37 @@
     </row>
     <row r="22" spans="2:15" ht="17.25" thickBot="1">
       <c r="B22" s="10"/>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="23"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+      <c r="O22" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="F17:O17"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F16:O16"/>
     <mergeCell ref="C21:O21"/>
     <mergeCell ref="C22:O22"/>
     <mergeCell ref="C10:I10"/>
@@ -4097,19 +4156,6 @@
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="F16:O16"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C9:O9"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C8:O8"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4123,46 +4169,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="C3" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="15"/>
+      <c r="C4" s="18"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -4180,8 +4226,8 @@
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>103</v>
+      <c r="C5" s="18" t="s">
+        <v>102</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -4198,7 +4244,7 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="6"/>
-      <c r="C6" s="15"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -4214,19 +4260,19 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="18" t="s">
         <v>16</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>17</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="28" t="s">
-        <v>38</v>
+      <c r="I7" s="19"/>
+      <c r="J7" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="K7" s="16"/>
       <c r="L7" s="16"/>
@@ -4236,14 +4282,14 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="15"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="28"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="15"/>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
@@ -4252,10 +4298,10 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -4272,7 +4318,7 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="15"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -4290,13 +4336,13 @@
       <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="15" t="s">
         <v>43</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28" t="s">
-        <v>44</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
@@ -4310,10 +4356,10 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -4328,13 +4374,13 @@
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>45</v>
+      <c r="C13" s="18" t="s">
+        <v>44</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28" t="s">
-        <v>44</v>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15" t="s">
+        <v>43</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
@@ -4350,10 +4396,10 @@
       <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="15"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -4366,10 +4412,10 @@
     </row>
     <row r="15" spans="2:15" ht="17.25" thickBot="1">
       <c r="B15" s="4"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="18"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -4382,27 +4428,27 @@
     </row>
     <row r="16" spans="2:15">
       <c r="B16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="21"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="21"/>
+      <c r="N16" s="21"/>
+      <c r="O16" s="22"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="6"/>
-      <c r="C17" s="15"/>
+      <c r="C17" s="18"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
@@ -4418,48 +4464,48 @@
     </row>
     <row r="18" spans="2:15" ht="17.25" thickBot="1">
       <c r="B18" s="10"/>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="23"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
+      <c r="O18" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C16:O16"/>
-    <mergeCell ref="C17:O17"/>
-    <mergeCell ref="C18:O18"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:O11"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="F12:O12"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="F13:O13"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="C9:O9"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="F11:O11"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C16:O16"/>
+    <mergeCell ref="C17:O17"/>
+    <mergeCell ref="C18:O18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4467,54 +4513,52 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBBC34AE-CE54-4DB4-B6C8-1E8F5594BE9D}">
-  <dimension ref="B1:O21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58695A09-AA77-4D28-9ABB-B6E5264761CD}">
+  <dimension ref="B1:O22"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
-    <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
+    <row r="1" spans="2:15" ht="17.25" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="C3" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="15" t="s">
-        <v>58</v>
-      </c>
+      <c r="C4" s="18"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -4529,8 +4573,12 @@
       <c r="O4" s="17"/>
     </row>
     <row r="5" spans="2:15">
-      <c r="B5" s="2"/>
-      <c r="C5" s="15"/>
+      <c r="B5" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>107</v>
+      </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -4545,11 +4593,9 @@
       <c r="O5" s="17"/>
     </row>
     <row r="6" spans="2:15">
-      <c r="B6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>55</v>
+      <c r="B6" s="6"/>
+      <c r="C6" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -4566,7 +4612,9 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="15"/>
+      <c r="C7" s="18" t="s">
+        <v>108</v>
+      </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -4581,35 +4629,33 @@
       <c r="O7" s="17"/>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="17"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="42"/>
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="15"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="28"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
@@ -4617,10 +4663,8 @@
       <c r="O9" s="17"/>
     </row>
     <row r="10" spans="2:15">
-      <c r="B10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="15"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -4635,8 +4679,434 @@
       <c r="O10" s="17"/>
     </row>
     <row r="11" spans="2:15">
+      <c r="B11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="17"/>
+    </row>
+    <row r="12" spans="2:15">
+      <c r="B12" s="6"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="17"/>
+    </row>
+    <row r="13" spans="2:15">
+      <c r="B13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+      <c r="O13" s="17"/>
+    </row>
+    <row r="14" spans="2:15">
+      <c r="B14" s="6"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="17"/>
+    </row>
+    <row r="15" spans="2:15">
+      <c r="B15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="17"/>
+    </row>
+    <row r="16" spans="2:15">
+      <c r="B16" s="6"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="17"/>
+    </row>
+    <row r="17" spans="2:15">
+      <c r="B17" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="16"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="17"/>
+    </row>
+    <row r="18" spans="2:15">
+      <c r="B18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="17"/>
+    </row>
+    <row r="19" spans="2:15" ht="17.25" thickBot="1">
+      <c r="B19" s="4"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="17"/>
+    </row>
+    <row r="20" spans="2:15">
+      <c r="B20" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="22"/>
+    </row>
+    <row r="21" spans="2:15">
+      <c r="B21" s="6"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="17"/>
+    </row>
+    <row r="22" spans="2:15" ht="17.25" thickBot="1">
+      <c r="B22" s="10"/>
+      <c r="C22" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+      <c r="O22" s="25"/>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="C22:O22"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F18:O18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="F19:O19"/>
+    <mergeCell ref="C20:O20"/>
+    <mergeCell ref="C21:O21"/>
+    <mergeCell ref="C13:O13"/>
+    <mergeCell ref="C14:O14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F16:O16"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:O17"/>
+    <mergeCell ref="C11:I11"/>
+    <mergeCell ref="J11:O11"/>
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="J12:O12"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBBC34AE-CE54-4DB4-B6C8-1E8F5594BE9D}">
+  <dimension ref="B1:O21"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetData>
+    <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
+    <row r="2" spans="2:15" ht="17.25" thickBot="1">
+      <c r="B2" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
+    </row>
+    <row r="3" spans="2:15">
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
+    </row>
+    <row r="4" spans="2:15">
+      <c r="B4" s="2"/>
+      <c r="C4" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="17"/>
+    </row>
+    <row r="5" spans="2:15">
+      <c r="B5" s="2"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="17"/>
+    </row>
+    <row r="6" spans="2:15">
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="17"/>
+    </row>
+    <row r="7" spans="2:15">
+      <c r="B7" s="6"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="17"/>
+    </row>
+    <row r="8" spans="2:15">
+      <c r="B8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="18"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="17"/>
+    </row>
+    <row r="9" spans="2:15">
+      <c r="B9" s="6"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="17"/>
+    </row>
+    <row r="10" spans="2:15">
+      <c r="B10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="17"/>
+    </row>
+    <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="15"/>
+      <c r="C11" s="18"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -4654,13 +5124,13 @@
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>65</v>
+      <c r="C12" s="18" t="s">
+        <v>64</v>
       </c>
       <c r="D12" s="16"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28" t="s">
-        <v>68</v>
+      <c r="E12" s="19"/>
+      <c r="F12" s="15" t="s">
+        <v>67</v>
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
@@ -4674,13 +5144,13 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="15" t="s">
-        <v>13</v>
+      <c r="C13" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28" t="s">
-        <v>67</v>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15" t="s">
+        <v>66</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
@@ -4694,13 +5164,13 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15" t="s">
         <v>66</v>
-      </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28" t="s">
-        <v>67</v>
       </c>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
@@ -4714,10 +5184,10 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="6"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="18"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -4732,13 +5202,13 @@
       <c r="B16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="15" t="s">
         <v>63</v>
-      </c>
-      <c r="D16" s="16"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="28" t="s">
-        <v>64</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -4754,10 +5224,10 @@
       <c r="B17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="15"/>
+      <c r="C17" s="18"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -4770,10 +5240,10 @@
     </row>
     <row r="18" spans="2:15" ht="17.25" thickBot="1">
       <c r="B18" s="4"/>
-      <c r="C18" s="15"/>
+      <c r="C18" s="18"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="28"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="15"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
@@ -4786,27 +5256,27 @@
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="20"/>
+        <v>35</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="22"/>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="6"/>
-      <c r="C20" s="15"/>
+      <c r="C20" s="18"/>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
@@ -4822,38 +5292,30 @@
     </row>
     <row r="21" spans="2:15" ht="17.25" thickBot="1">
       <c r="B21" s="10"/>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="23"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="J9:O9"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:O11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:O12"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="F14:O14"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F18:O18"/>
     <mergeCell ref="C19:O19"/>
     <mergeCell ref="C20:O20"/>
     <mergeCell ref="C21:O21"/>
@@ -4863,65 +5325,73 @@
     <mergeCell ref="F16:O16"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="F14:O14"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="F18:O18"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="J9:O9"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="F12:O12"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C7:O7"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF70DE72-D01A-446C-8863-B94658AF56DE}">
   <dimension ref="B1:O20"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B2" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20"/>
+      <c r="C3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="15"/>
+      <c r="C4" s="18"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -4937,7 +5407,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="15"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -4955,7 +5425,7 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="15"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -4971,7 +5441,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="15"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -4987,16 +5457,16 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="15"/>
+        <v>15</v>
+      </c>
+      <c r="C8" s="18"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="28"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="15"/>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
@@ -5005,14 +5475,14 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="15"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="28"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="15"/>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
@@ -5021,9 +5491,9 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="C10" s="18"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -5039,7 +5509,7 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="15"/>
+      <c r="C11" s="18"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -5057,10 +5527,10 @@
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="15"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -5073,10 +5543,10 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="15"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
@@ -5091,10 +5561,10 @@
       <c r="B14" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="15"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -5109,10 +5579,10 @@
       <c r="B15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
+      <c r="C15" s="18"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -5125,10 +5595,10 @@
     </row>
     <row r="16" spans="2:15" ht="17.25" thickBot="1">
       <c r="B16" s="4"/>
-      <c r="C16" s="15"/>
+      <c r="C16" s="18"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="28"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -5141,27 +5611,27 @@
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="19"/>
-      <c r="O17" s="20"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+      <c r="O17" s="22"/>
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="6"/>
-      <c r="C18" s="15"/>
+      <c r="C18" s="18"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
@@ -5177,21 +5647,21 @@
     </row>
     <row r="19" spans="2:15" ht="17.25" thickBot="1">
       <c r="B19" s="10"/>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="23"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="24"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="24"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="25"/>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="14"/>
@@ -5213,6 +5683,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="F14:O14"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="F16:O16"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C4:O4"/>
     <mergeCell ref="C17:O17"/>
     <mergeCell ref="C18:O18"/>
     <mergeCell ref="C19:O19"/>
@@ -5229,15 +5708,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F12:O12"/>
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="F14:O14"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="F16:O16"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:O11"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C4:O4"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feature : Inventroy 컴포넌트 추가
* PlayerController의 컴포넌트 제작
* Strcut 재정의 2차 배열로 Slot 제작
* ItemID가 키 값인 Map으로 Slot을 찾도록 구현
* 빈 슬롯 탐색 알고리즘 : O(N^2)

* 필드의 아이템 충돌하고 선택된 아이템을 인벤토리로 획득하고 Actor가 사라지는 것까지 Test
</commit_message>
<xml_diff>
--- a/코드 파일 기술서.xlsx
+++ b/코드 파일 기술서.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\source\repos\Unreal\UE5\TopDownPortfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62A5BF95-78B4-4B21-89AD-EC09535141E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD3C753-441D-4881-9FF2-3258CAE928A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="6" xr2:uid="{D21DC332-3B34-4EF0-AFA4-A1E5433A082F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="726" activeTab="1" xr2:uid="{D21DC332-3B34-4EF0-AFA4-A1E5433A082F}"/>
   </bookViews>
   <sheets>
     <sheet name="코드 작성 양식" sheetId="2" r:id="rId1"/>
@@ -1110,19 +1110,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1152,19 +1146,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1183,6 +1168,21 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1536,22 +1536,22 @@
   <sheetData>
     <row r="1" spans="2:18" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:18" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
       <c r="Q2" s="1" t="s">
         <v>38</v>
       </c>
@@ -1563,21 +1563,21 @@
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
       <c r="Q3" s="1"/>
       <c r="R3" t="s">
         <v>39</v>
@@ -1585,7 +1585,7 @@
     </row>
     <row r="4" spans="2:18">
       <c r="B4" s="2"/>
-      <c r="C4" s="18"/>
+      <c r="C4" s="15"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -1603,7 +1603,7 @@
       <c r="B5" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="15" t="s">
         <v>106</v>
       </c>
       <c r="D5" s="16"/>
@@ -1621,7 +1621,7 @@
     </row>
     <row r="6" spans="2:18">
       <c r="B6" s="6"/>
-      <c r="C6" s="18"/>
+      <c r="C6" s="15"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -1639,7 +1639,7 @@
       <c r="B7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="16"/>
@@ -1647,8 +1647,8 @@
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="15" t="s">
+      <c r="I7" s="27"/>
+      <c r="J7" s="28" t="s">
         <v>37</v>
       </c>
       <c r="K7" s="16"/>
@@ -1659,14 +1659,14 @@
     </row>
     <row r="8" spans="2:18">
       <c r="B8" s="6"/>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="15"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="28"/>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
@@ -1677,7 +1677,7 @@
       <c r="B9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="16"/>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="10" spans="2:18">
       <c r="B10" s="6"/>
-      <c r="C10" s="18"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -1713,12 +1713,12 @@
       <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="15" t="s">
         <v>42</v>
       </c>
       <c r="D11" s="16"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="15" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G11" s="16"/>
@@ -1733,10 +1733,10 @@
     </row>
     <row r="12" spans="2:18">
       <c r="B12" s="6"/>
-      <c r="C12" s="18"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="15"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -1751,12 +1751,12 @@
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15" t="s">
+      <c r="E13" s="27"/>
+      <c r="F13" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G13" s="16"/>
@@ -1773,10 +1773,10 @@
       <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="18"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -1789,10 +1789,10 @@
     </row>
     <row r="15" spans="2:18" ht="17.25" thickBot="1">
       <c r="B15" s="4"/>
-      <c r="C15" s="18"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -1807,25 +1807,25 @@
       <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="22"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="20"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="6"/>
-      <c r="C17" s="18"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
@@ -1841,24 +1841,32 @@
     </row>
     <row r="18" spans="2:15" ht="17.25" thickBot="1">
       <c r="B18" s="10"/>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
-      <c r="L18" s="24"/>
-      <c r="M18" s="24"/>
-      <c r="N18" s="24"/>
-      <c r="O18" s="25"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:O11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="F12:O12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
     <mergeCell ref="C17:O17"/>
     <mergeCell ref="C16:O16"/>
     <mergeCell ref="C18:O18"/>
@@ -1875,14 +1883,6 @@
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
     <mergeCell ref="C15:E15"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="F11:O11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:O12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1896,46 +1896,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15" ht="15" customHeight="1">
       <c r="B4" s="2"/>
-      <c r="C4" s="18"/>
+      <c r="C4" s="15"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -1953,7 +1953,7 @@
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="15" t="s">
         <v>47</v>
       </c>
       <c r="D5" s="16"/>
@@ -1971,7 +1971,7 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="6"/>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>48</v>
       </c>
       <c r="D6" s="16"/>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18"/>
+      <c r="C7" s="15"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -2007,14 +2007,14 @@
       <c r="B8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="15" t="s">
+      <c r="I8" s="27"/>
+      <c r="J8" s="28" t="s">
         <v>37</v>
       </c>
       <c r="K8" s="16"/>
@@ -2025,14 +2025,14 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="18"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="15"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="28"/>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
@@ -2043,7 +2043,7 @@
       <c r="B10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="15" t="s">
         <v>50</v>
       </c>
       <c r="D10" s="16"/>
@@ -2061,7 +2061,7 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="18"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -2079,12 +2079,12 @@
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D12" s="16"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="15" t="s">
+      <c r="E12" s="27"/>
+      <c r="F12" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G12" s="16"/>
@@ -2099,10 +2099,10 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="18"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
@@ -2115,10 +2115,10 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="18"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -2133,12 +2133,12 @@
       <c r="B15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15" t="s">
+      <c r="E15" s="27"/>
+      <c r="F15" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G15" s="16"/>
@@ -2155,10 +2155,10 @@
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="18"/>
+      <c r="C16" s="15"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="15"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -2171,10 +2171,10 @@
     </row>
     <row r="17" spans="2:15" ht="17.25" thickBot="1">
       <c r="B17" s="4"/>
-      <c r="C17" s="18"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="15"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -2189,25 +2189,25 @@
       <c r="B18" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="22"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="20"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="6"/>
-      <c r="C19" s="18"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
@@ -2223,32 +2223,29 @@
     </row>
     <row r="20" spans="2:15" ht="17.25" thickBot="1">
       <c r="B20" s="10"/>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
-      <c r="O20" s="25"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:O17"/>
+    <mergeCell ref="C18:O18"/>
+    <mergeCell ref="C19:O19"/>
+    <mergeCell ref="C20:O20"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F16:O16"/>
     <mergeCell ref="C9:I9"/>
@@ -2263,11 +2260,14 @@
     <mergeCell ref="F14:O14"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C18:O18"/>
-    <mergeCell ref="C19:O19"/>
-    <mergeCell ref="C20:O20"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2281,46 +2281,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="15" t="s">
         <v>85</v>
       </c>
       <c r="D4" s="16"/>
@@ -2338,7 +2338,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="18"/>
+      <c r="C5" s="15"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -2356,7 +2356,7 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>59</v>
       </c>
       <c r="D6" s="16"/>
@@ -2374,7 +2374,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>82</v>
       </c>
       <c r="D7" s="16"/>
@@ -2392,7 +2392,7 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -2410,7 +2410,7 @@
       <c r="B9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="16"/>
@@ -2418,8 +2418,8 @@
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="15" t="s">
+      <c r="I9" s="27"/>
+      <c r="J9" s="28" t="s">
         <v>37</v>
       </c>
       <c r="K9" s="16"/>
@@ -2430,14 +2430,14 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="18"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="15"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="28"/>
       <c r="K10" s="16"/>
       <c r="L10" s="16"/>
       <c r="M10" s="16"/>
@@ -2448,7 +2448,7 @@
       <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="15" t="s">
         <v>60</v>
       </c>
       <c r="D11" s="16"/>
@@ -2466,7 +2466,7 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="18"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
@@ -2484,12 +2484,12 @@
       <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>79</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15" t="s">
+      <c r="E13" s="27"/>
+      <c r="F13" s="28" t="s">
         <v>71</v>
       </c>
       <c r="G13" s="16"/>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="18"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -2522,12 +2522,12 @@
       <c r="B15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>80</v>
       </c>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15" t="s">
+      <c r="E15" s="27"/>
+      <c r="F15" s="28" t="s">
         <v>81</v>
       </c>
       <c r="G15" s="16"/>
@@ -2544,10 +2544,10 @@
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="18"/>
+      <c r="C16" s="15"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="15"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -2560,10 +2560,10 @@
     </row>
     <row r="17" spans="2:15" ht="17.25" thickBot="1">
       <c r="B17" s="4"/>
-      <c r="C17" s="18"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="15"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -2578,23 +2578,23 @@
       <c r="B18" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="20"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="22"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="20"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="6"/>
-      <c r="C19" s="18"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
@@ -2610,64 +2610,64 @@
     </row>
     <row r="20" spans="2:15" ht="17.25" thickBot="1">
       <c r="B20" s="10"/>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
-      <c r="O20" s="25"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="23"/>
     </row>
     <row r="22" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="23" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
-      <c r="N23" s="27"/>
-      <c r="O23" s="28"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="25"/>
+      <c r="N23" s="25"/>
+      <c r="O23" s="26"/>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="21"/>
-      <c r="O24" s="22"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19"/>
+      <c r="O24" s="20"/>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2"/>
-      <c r="C25" s="18"/>
+      <c r="C25" s="15"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
@@ -2683,7 +2683,7 @@
     </row>
     <row r="26" spans="2:15">
       <c r="B26" s="2"/>
-      <c r="C26" s="18"/>
+      <c r="C26" s="15"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
@@ -2701,7 +2701,7 @@
       <c r="B27" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C27" s="18"/>
+      <c r="C27" s="15"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
@@ -2717,7 +2717,7 @@
     </row>
     <row r="28" spans="2:15">
       <c r="B28" s="6"/>
-      <c r="C28" s="18"/>
+      <c r="C28" s="15"/>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
@@ -2735,7 +2735,7 @@
       <c r="B29" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="15" t="s">
         <v>77</v>
       </c>
       <c r="D29" s="16"/>
@@ -2743,8 +2743,8 @@
       <c r="F29" s="16"/>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="15"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="28"/>
       <c r="K29" s="16"/>
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
@@ -2753,7 +2753,7 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="6"/>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="15" t="s">
         <v>78</v>
       </c>
       <c r="D30" s="16"/>
@@ -2761,8 +2761,8 @@
       <c r="F30" s="16"/>
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="15"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="28"/>
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
@@ -2771,14 +2771,14 @@
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="6"/>
-      <c r="C31" s="18"/>
+      <c r="C31" s="15"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="15"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="28"/>
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
@@ -2789,7 +2789,7 @@
       <c r="B32" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C32" s="18"/>
+      <c r="C32" s="15"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
@@ -2805,7 +2805,7 @@
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="6"/>
-      <c r="C33" s="18"/>
+      <c r="C33" s="15"/>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
       <c r="F33" s="16"/>
@@ -2823,12 +2823,12 @@
       <c r="B34" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="15" t="s">
         <v>72</v>
       </c>
       <c r="D34" s="16"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="15" t="s">
+      <c r="E34" s="27"/>
+      <c r="F34" s="28" t="s">
         <v>74</v>
       </c>
       <c r="G34" s="16"/>
@@ -2843,12 +2843,12 @@
     </row>
     <row r="35" spans="2:15">
       <c r="B35" s="6"/>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="15" t="s">
         <v>72</v>
       </c>
       <c r="D35" s="16"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="15" t="s">
+      <c r="E35" s="27"/>
+      <c r="F35" s="28" t="s">
         <v>73</v>
       </c>
       <c r="G35" s="16"/>
@@ -2863,12 +2863,12 @@
     </row>
     <row r="36" spans="2:15">
       <c r="B36" s="6"/>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="15" t="s">
         <v>75</v>
       </c>
       <c r="D36" s="16"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="15" t="s">
+      <c r="E36" s="27"/>
+      <c r="F36" s="28" t="s">
         <v>76</v>
       </c>
       <c r="G36" s="16"/>
@@ -2883,10 +2883,10 @@
     </row>
     <row r="37" spans="2:15">
       <c r="B37" s="6"/>
-      <c r="C37" s="18"/>
+      <c r="C37" s="15"/>
       <c r="D37" s="16"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="15"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="28"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
       <c r="I37" s="16"/>
@@ -2901,12 +2901,12 @@
       <c r="B38" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="C38" s="15" t="s">
         <v>83</v>
       </c>
       <c r="D38" s="16"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="15" t="s">
+      <c r="E38" s="27"/>
+      <c r="F38" s="28" t="s">
         <v>84</v>
       </c>
       <c r="G38" s="16"/>
@@ -2923,10 +2923,10 @@
       <c r="B39" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="18"/>
+      <c r="C39" s="15"/>
       <c r="D39" s="16"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="15"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="28"/>
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
@@ -2939,10 +2939,10 @@
     </row>
     <row r="40" spans="2:15" ht="17.25" thickBot="1">
       <c r="B40" s="4"/>
-      <c r="C40" s="18"/>
+      <c r="C40" s="15"/>
       <c r="D40" s="16"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="15"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="28"/>
       <c r="G40" s="16"/>
       <c r="H40" s="16"/>
       <c r="I40" s="16"/>
@@ -2957,23 +2957,23 @@
       <c r="B41" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C41" s="20"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="21"/>
-      <c r="J41" s="21"/>
-      <c r="K41" s="21"/>
-      <c r="L41" s="21"/>
-      <c r="M41" s="21"/>
-      <c r="N41" s="21"/>
-      <c r="O41" s="22"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
+      <c r="N41" s="19"/>
+      <c r="O41" s="20"/>
     </row>
     <row r="42" spans="2:15">
       <c r="B42" s="6"/>
-      <c r="C42" s="18"/>
+      <c r="C42" s="15"/>
       <c r="D42" s="16"/>
       <c r="E42" s="16"/>
       <c r="F42" s="16"/>
@@ -2989,52 +2989,37 @@
     </row>
     <row r="43" spans="2:15" ht="17.25" thickBot="1">
       <c r="B43" s="10"/>
-      <c r="C43" s="23" t="s">
+      <c r="C43" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-      <c r="G43" s="24"/>
-      <c r="H43" s="24"/>
-      <c r="I43" s="24"/>
-      <c r="J43" s="24"/>
-      <c r="K43" s="24"/>
-      <c r="L43" s="24"/>
-      <c r="M43" s="24"/>
-      <c r="N43" s="24"/>
-      <c r="O43" s="25"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="22"/>
+      <c r="J43" s="22"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="22"/>
+      <c r="M43" s="22"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="57">
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="F35:O35"/>
-    <mergeCell ref="C30:I30"/>
-    <mergeCell ref="J30:O30"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="F40:O40"/>
-    <mergeCell ref="C31:I31"/>
-    <mergeCell ref="J31:O31"/>
-    <mergeCell ref="C32:O32"/>
-    <mergeCell ref="C33:O33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="F34:O34"/>
-    <mergeCell ref="C41:O41"/>
-    <mergeCell ref="C42:O42"/>
-    <mergeCell ref="C43:O43"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="F36:O36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="F37:O37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="F38:O38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="F39:O39"/>
-    <mergeCell ref="C24:O24"/>
-    <mergeCell ref="C25:O25"/>
-    <mergeCell ref="C26:O26"/>
-    <mergeCell ref="C27:O27"/>
-    <mergeCell ref="C28:O28"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="J10:O10"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="J9:O9"/>
+    <mergeCell ref="C11:O11"/>
     <mergeCell ref="C29:I29"/>
     <mergeCell ref="J29:O29"/>
     <mergeCell ref="B23:O23"/>
@@ -3051,19 +3036,34 @@
     <mergeCell ref="C12:O12"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="J9:O9"/>
-    <mergeCell ref="C11:O11"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C10:I10"/>
-    <mergeCell ref="J10:O10"/>
+    <mergeCell ref="C24:O24"/>
+    <mergeCell ref="C25:O25"/>
+    <mergeCell ref="C26:O26"/>
+    <mergeCell ref="C27:O27"/>
+    <mergeCell ref="C28:O28"/>
+    <mergeCell ref="C41:O41"/>
+    <mergeCell ref="C42:O42"/>
+    <mergeCell ref="C43:O43"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="F36:O36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="F37:O37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="F38:O38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="F39:O39"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:O35"/>
+    <mergeCell ref="C30:I30"/>
+    <mergeCell ref="J30:O30"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="F40:O40"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="J31:O31"/>
+    <mergeCell ref="C32:O32"/>
+    <mergeCell ref="C33:O33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="F34:O34"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3081,46 +3081,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="31"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="37"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="5"/>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="15" t="s">
         <v>31</v>
       </c>
       <c r="D4" s="16"/>
@@ -3138,43 +3138,43 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="5"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="31"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="37"/>
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="32"/>
-      <c r="M6" s="32"/>
-      <c r="N6" s="32"/>
-      <c r="O6" s="33"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="38"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="39"/>
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="16"/>
@@ -3192,7 +3192,7 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -3210,7 +3210,7 @@
       <c r="B9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="15" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="16"/>
@@ -3218,7 +3218,7 @@
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="19"/>
+      <c r="I9" s="27"/>
       <c r="J9" s="16" t="s">
         <v>21</v>
       </c>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="15" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="16"/>
@@ -3238,7 +3238,7 @@
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="19"/>
+      <c r="I10" s="27"/>
       <c r="J10" s="16" t="s">
         <v>24</v>
       </c>
@@ -3250,7 +3250,7 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="15" t="s">
         <v>25</v>
       </c>
       <c r="D11" s="16"/>
@@ -3258,7 +3258,7 @@
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="19"/>
+      <c r="I11" s="27"/>
       <c r="J11" s="16" t="s">
         <v>20</v>
       </c>
@@ -3270,13 +3270,13 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="18"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
-      <c r="I12" s="19"/>
+      <c r="I12" s="27"/>
       <c r="J12" s="16"/>
       <c r="K12" s="16"/>
       <c r="L12" s="16"/>
@@ -3288,7 +3288,7 @@
       <c r="B13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>32</v>
       </c>
       <c r="D13" s="16"/>
@@ -3306,7 +3306,7 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="15" t="s">
         <v>30</v>
       </c>
       <c r="D14" s="16"/>
@@ -3324,7 +3324,7 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="6"/>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>33</v>
       </c>
       <c r="D15" s="16"/>
@@ -3342,7 +3342,7 @@
     </row>
     <row r="16" spans="2:15">
       <c r="B16" s="6"/>
-      <c r="C16" s="18"/>
+      <c r="C16" s="15"/>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
@@ -3383,7 +3383,7 @@
       <c r="C18" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="28" t="s">
         <v>13</v>
       </c>
       <c r="E18" s="16"/>
@@ -3403,7 +3403,7 @@
       <c r="C19" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="28" t="s">
         <v>14</v>
       </c>
       <c r="E19" s="16"/>
@@ -3420,7 +3420,7 @@
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="6"/>
-      <c r="D20" s="15"/>
+      <c r="D20" s="28"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
       <c r="G20" s="16"/>
@@ -3436,7 +3436,7 @@
     <row r="21" spans="2:15">
       <c r="B21" s="6"/>
       <c r="C21" s="7"/>
-      <c r="D21" s="15"/>
+      <c r="D21" s="28"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
@@ -3456,7 +3456,7 @@
       <c r="C22" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="28" t="s">
         <v>34</v>
       </c>
       <c r="E22" s="16"/>
@@ -3476,7 +3476,7 @@
       <c r="C23" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E23" s="16"/>
@@ -3496,7 +3496,7 @@
       <c r="C24" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="28" t="s">
         <v>28</v>
       </c>
       <c r="E24" s="16"/>
@@ -3516,7 +3516,7 @@
       <c r="C25" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="28" t="s">
         <v>27</v>
       </c>
       <c r="E25" s="16"/>
@@ -3550,153 +3550,164 @@
     <row r="27" spans="2:15" ht="17.25" thickBot="1">
       <c r="B27" s="4"/>
       <c r="C27" s="8"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
-      <c r="J27" s="24"/>
-      <c r="K27" s="24"/>
-      <c r="L27" s="24"/>
-      <c r="M27" s="24"/>
-      <c r="N27" s="24"/>
-      <c r="O27" s="25"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+      <c r="M27" s="22"/>
+      <c r="N27" s="22"/>
+      <c r="O27" s="23"/>
     </row>
     <row r="28" spans="2:15">
       <c r="B28" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="37" t="s">
+      <c r="C28" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="38"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="38"/>
-      <c r="J28" s="38"/>
-      <c r="K28" s="38"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="38"/>
-      <c r="N28" s="38"/>
-      <c r="O28" s="39"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="33"/>
+      <c r="M28" s="33"/>
+      <c r="N28" s="33"/>
+      <c r="O28" s="34"/>
     </row>
     <row r="29" spans="2:15">
       <c r="B29" s="11"/>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="D29" s="35"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35"/>
-      <c r="K29" s="35"/>
-      <c r="L29" s="35"/>
-      <c r="M29" s="35"/>
-      <c r="N29" s="35"/>
-      <c r="O29" s="36"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+      <c r="O29" s="31"/>
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="11"/>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="35"/>
-      <c r="H30" s="35"/>
-      <c r="I30" s="35"/>
-      <c r="J30" s="35"/>
-      <c r="K30" s="35"/>
-      <c r="L30" s="35"/>
-      <c r="M30" s="35"/>
-      <c r="N30" s="35"/>
-      <c r="O30" s="36"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="30"/>
+      <c r="O30" s="31"/>
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="11"/>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
-      <c r="K31" s="35"/>
-      <c r="L31" s="35"/>
-      <c r="M31" s="35"/>
-      <c r="N31" s="35"/>
-      <c r="O31" s="36"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
+      <c r="O31" s="31"/>
     </row>
     <row r="32" spans="2:15">
       <c r="B32" s="11"/>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="35"/>
-      <c r="J32" s="35"/>
-      <c r="K32" s="35"/>
-      <c r="L32" s="35"/>
-      <c r="M32" s="35"/>
-      <c r="N32" s="35"/>
-      <c r="O32" s="36"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
+      <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
+      <c r="M32" s="30"/>
+      <c r="N32" s="30"/>
+      <c r="O32" s="31"/>
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="11"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="35"/>
-      <c r="K33" s="35"/>
-      <c r="L33" s="35"/>
-      <c r="M33" s="35"/>
-      <c r="N33" s="35"/>
-      <c r="O33" s="36"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
+      <c r="K33" s="30"/>
+      <c r="L33" s="30"/>
+      <c r="M33" s="30"/>
+      <c r="N33" s="30"/>
+      <c r="O33" s="31"/>
     </row>
     <row r="34" spans="2:15" ht="17.25" thickBot="1">
       <c r="B34" s="10"/>
-      <c r="C34" s="23" t="s">
+      <c r="C34" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-      <c r="L34" s="24"/>
-      <c r="M34" s="24"/>
-      <c r="N34" s="24"/>
-      <c r="O34" s="25"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="22"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+      <c r="M34" s="22"/>
+      <c r="N34" s="22"/>
+      <c r="O34" s="23"/>
     </row>
     <row r="40" spans="2:15" ht="17.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="C31:O31"/>
-    <mergeCell ref="C29:O29"/>
-    <mergeCell ref="C30:O30"/>
-    <mergeCell ref="C32:O32"/>
-    <mergeCell ref="C28:O28"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C13:O13"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="D26:O26"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="D19:O19"/>
+    <mergeCell ref="D24:O24"/>
+    <mergeCell ref="D21:O21"/>
+    <mergeCell ref="D20:O20"/>
+    <mergeCell ref="C16:O16"/>
+    <mergeCell ref="D17:O17"/>
+    <mergeCell ref="D18:O18"/>
     <mergeCell ref="C34:O34"/>
     <mergeCell ref="C33:O33"/>
     <mergeCell ref="C9:I9"/>
@@ -3713,22 +3724,11 @@
     <mergeCell ref="D23:O23"/>
     <mergeCell ref="D22:O22"/>
     <mergeCell ref="D25:O25"/>
-    <mergeCell ref="D26:O26"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="D19:O19"/>
-    <mergeCell ref="D24:O24"/>
-    <mergeCell ref="D21:O21"/>
-    <mergeCell ref="D20:O20"/>
-    <mergeCell ref="C16:O16"/>
-    <mergeCell ref="D17:O17"/>
-    <mergeCell ref="D18:O18"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C13:O13"/>
-    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C31:O31"/>
+    <mergeCell ref="C29:O29"/>
+    <mergeCell ref="C30:O30"/>
+    <mergeCell ref="C32:O32"/>
+    <mergeCell ref="C28:O28"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3742,46 +3742,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="15" t="s">
         <v>99</v>
       </c>
       <c r="D4" s="16"/>
@@ -3799,7 +3799,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="18"/>
+      <c r="C5" s="15"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -3817,7 +3817,7 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>92</v>
       </c>
       <c r="D6" s="16"/>
@@ -3835,7 +3835,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>93</v>
       </c>
       <c r="D7" s="16"/>
@@ -3853,7 +3853,7 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -3869,7 +3869,7 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="18"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
@@ -3887,7 +3887,7 @@
       <c r="B10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="16"/>
@@ -3895,8 +3895,8 @@
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="15" t="s">
+      <c r="I10" s="27"/>
+      <c r="J10" s="28" t="s">
         <v>37</v>
       </c>
       <c r="K10" s="16"/>
@@ -3907,14 +3907,14 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="18"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="15"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
       <c r="K11" s="16"/>
       <c r="L11" s="16"/>
       <c r="M11" s="16"/>
@@ -3925,7 +3925,7 @@
       <c r="B12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="15" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="16"/>
@@ -3943,7 +3943,7 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="18"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
@@ -3961,12 +3961,12 @@
       <c r="B14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="15" t="s">
         <v>94</v>
       </c>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15" t="s">
+      <c r="E14" s="27"/>
+      <c r="F14" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G14" s="16"/>
@@ -3981,10 +3981,10 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="6"/>
-      <c r="C15" s="18"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -3999,12 +3999,12 @@
       <c r="B16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="15" t="s">
         <v>98</v>
       </c>
       <c r="D16" s="16"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="15" t="s">
+      <c r="E16" s="27"/>
+      <c r="F16" s="28" t="s">
         <v>96</v>
       </c>
       <c r="G16" s="16"/>
@@ -4021,12 +4021,12 @@
       <c r="B17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="15" t="s">
         <v>95</v>
       </c>
       <c r="D17" s="16"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="15" t="s">
+      <c r="E17" s="27"/>
+      <c r="F17" s="28" t="s">
         <v>97</v>
       </c>
       <c r="G17" s="16"/>
@@ -4041,10 +4041,10 @@
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="3"/>
-      <c r="C18" s="18"/>
+      <c r="C18" s="15"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="15"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="28"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
@@ -4057,10 +4057,10 @@
     </row>
     <row r="19" spans="2:15" ht="17.25" thickBot="1">
       <c r="B19" s="4"/>
-      <c r="C19" s="18"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="16"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="15"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
@@ -4075,25 +4075,25 @@
       <c r="B20" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="21"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="22"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="20"/>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="6"/>
-      <c r="C21" s="18"/>
+      <c r="C21" s="15"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
@@ -4109,37 +4109,24 @@
     </row>
     <row r="22" spans="2:15" ht="17.25" thickBot="1">
       <c r="B22" s="10"/>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="24"/>
-      <c r="N22" s="24"/>
-      <c r="O22" s="25"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C9:O9"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C7:O7"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="F16:O16"/>
     <mergeCell ref="C21:O21"/>
     <mergeCell ref="C22:O22"/>
     <mergeCell ref="C10:I10"/>
@@ -4156,6 +4143,19 @@
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="F14:O14"/>
     <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:O17"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F16:O16"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C8:O8"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4169,46 +4169,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="18"/>
+      <c r="C4" s="15"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -4226,7 +4226,7 @@
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="15" t="s">
         <v>102</v>
       </c>
       <c r="D5" s="16"/>
@@ -4244,7 +4244,7 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="6"/>
-      <c r="C6" s="18"/>
+      <c r="C6" s="15"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -4262,7 +4262,7 @@
       <c r="B7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="16"/>
@@ -4270,8 +4270,8 @@
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="15" t="s">
+      <c r="I7" s="27"/>
+      <c r="J7" s="28" t="s">
         <v>37</v>
       </c>
       <c r="K7" s="16"/>
@@ -4282,14 +4282,14 @@
     </row>
     <row r="8" spans="2:15">
       <c r="B8" s="6"/>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="15"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="28"/>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
@@ -4300,7 +4300,7 @@
       <c r="B9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="16"/>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="18"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -4336,12 +4336,12 @@
       <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="15" t="s">
         <v>42</v>
       </c>
       <c r="D11" s="16"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="15" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G11" s="16"/>
@@ -4356,10 +4356,10 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="18"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="15"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -4374,12 +4374,12 @@
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15" t="s">
+      <c r="E13" s="27"/>
+      <c r="F13" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G13" s="16"/>
@@ -4396,10 +4396,10 @@
       <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="18"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -4412,10 +4412,10 @@
     </row>
     <row r="15" spans="2:15" ht="17.25" thickBot="1">
       <c r="B15" s="4"/>
-      <c r="C15" s="18"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -4430,25 +4430,25 @@
       <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="22"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="20"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="6"/>
-      <c r="C17" s="18"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
@@ -4464,24 +4464,41 @@
     </row>
     <row r="18" spans="2:15" ht="17.25" thickBot="1">
       <c r="B18" s="10"/>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
-      <c r="L18" s="24"/>
-      <c r="M18" s="24"/>
-      <c r="N18" s="24"/>
-      <c r="O18" s="25"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="C16:O16"/>
+    <mergeCell ref="C17:O17"/>
+    <mergeCell ref="C18:O18"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="F12:O12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="F14:O14"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:O11"/>
     <mergeCell ref="C7:I7"/>
     <mergeCell ref="J7:O7"/>
     <mergeCell ref="B2:O2"/>
@@ -4489,23 +4506,6 @@
     <mergeCell ref="C4:O4"/>
     <mergeCell ref="C5:O5"/>
     <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="C9:O9"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="F11:O11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:O12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="F14:O14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="C16:O16"/>
-    <mergeCell ref="C17:O17"/>
-    <mergeCell ref="C18:O18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4519,46 +4519,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="18"/>
+      <c r="C4" s="15"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -4576,7 +4576,7 @@
       <c r="B5" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="15" t="s">
         <v>107</v>
       </c>
       <c r="D5" s="16"/>
@@ -4594,7 +4594,7 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="6"/>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>110</v>
       </c>
       <c r="D6" s="16"/>
@@ -4612,7 +4612,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>108</v>
       </c>
       <c r="D7" s="16"/>
@@ -4648,7 +4648,7 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="18"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
@@ -4664,7 +4664,7 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="6"/>
-      <c r="C10" s="18"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -4682,7 +4682,7 @@
       <c r="B11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="16"/>
@@ -4690,8 +4690,8 @@
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="15" t="s">
+      <c r="I11" s="27"/>
+      <c r="J11" s="28" t="s">
         <v>37</v>
       </c>
       <c r="K11" s="16"/>
@@ -4702,14 +4702,14 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="6"/>
-      <c r="C12" s="18"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="15"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
       <c r="K12" s="16"/>
       <c r="L12" s="16"/>
       <c r="M12" s="16"/>
@@ -4720,7 +4720,7 @@
       <c r="B13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>19</v>
       </c>
       <c r="D13" s="16"/>
@@ -4738,7 +4738,7 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="18"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
@@ -4756,12 +4756,12 @@
       <c r="B15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>42</v>
       </c>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15" t="s">
+      <c r="E15" s="27"/>
+      <c r="F15" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G15" s="16"/>
@@ -4776,10 +4776,10 @@
     </row>
     <row r="16" spans="2:15">
       <c r="B16" s="6"/>
-      <c r="C16" s="18"/>
+      <c r="C16" s="15"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="15"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -4794,12 +4794,12 @@
       <c r="B17" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D17" s="16"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="15" t="s">
+      <c r="E17" s="27"/>
+      <c r="F17" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G17" s="16"/>
@@ -4816,10 +4816,10 @@
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="18"/>
+      <c r="C18" s="15"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="15"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="28"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
@@ -4832,10 +4832,10 @@
     </row>
     <row r="19" spans="2:15" ht="17.25" thickBot="1">
       <c r="B19" s="4"/>
-      <c r="C19" s="18"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="16"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="15"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
@@ -4850,25 +4850,25 @@
       <c r="B20" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="21"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="22"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="20"/>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="6"/>
-      <c r="C21" s="18"/>
+      <c r="C21" s="15"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
@@ -4884,24 +4884,36 @@
     </row>
     <row r="22" spans="2:15" ht="17.25" thickBot="1">
       <c r="B22" s="10"/>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="24"/>
-      <c r="N22" s="24"/>
-      <c r="O22" s="25"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:O17"/>
+    <mergeCell ref="C11:I11"/>
+    <mergeCell ref="J11:O11"/>
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="F16:O16"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C10:O10"/>
     <mergeCell ref="C22:O22"/>
     <mergeCell ref="C8:O8"/>
     <mergeCell ref="C6:O6"/>
@@ -4918,18 +4930,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="F15:O15"/>
     <mergeCell ref="C16:E16"/>
-    <mergeCell ref="F16:O16"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C11:I11"/>
-    <mergeCell ref="J11:O11"/>
-    <mergeCell ref="C12:I12"/>
-    <mergeCell ref="J12:O12"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4943,46 +4943,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="15" t="s">
         <v>57</v>
       </c>
       <c r="D4" s="16"/>
@@ -5000,7 +5000,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="18"/>
+      <c r="C5" s="15"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -5018,7 +5018,7 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>54</v>
       </c>
       <c r="D6" s="16"/>
@@ -5036,7 +5036,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18"/>
+      <c r="C7" s="15"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -5054,14 +5054,14 @@
       <c r="B8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="15" t="s">
+      <c r="I8" s="27"/>
+      <c r="J8" s="28" t="s">
         <v>61</v>
       </c>
       <c r="K8" s="16"/>
@@ -5072,14 +5072,14 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="18"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="15"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="28"/>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
@@ -5090,7 +5090,7 @@
       <c r="B10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="18"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -5106,7 +5106,7 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="18"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -5124,12 +5124,12 @@
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="15" t="s">
         <v>64</v>
       </c>
       <c r="D12" s="16"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="15" t="s">
+      <c r="E12" s="27"/>
+      <c r="F12" s="28" t="s">
         <v>67</v>
       </c>
       <c r="G12" s="16"/>
@@ -5144,12 +5144,12 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15" t="s">
+      <c r="E13" s="27"/>
+      <c r="F13" s="28" t="s">
         <v>66</v>
       </c>
       <c r="G13" s="16"/>
@@ -5164,12 +5164,12 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="6"/>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="15" t="s">
         <v>65</v>
       </c>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15" t="s">
+      <c r="E14" s="27"/>
+      <c r="F14" s="28" t="s">
         <v>66</v>
       </c>
       <c r="G14" s="16"/>
@@ -5184,10 +5184,10 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="6"/>
-      <c r="C15" s="18"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -5202,12 +5202,12 @@
       <c r="B16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="15" t="s">
         <v>62</v>
       </c>
       <c r="D16" s="16"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="15" t="s">
+      <c r="E16" s="27"/>
+      <c r="F16" s="28" t="s">
         <v>63</v>
       </c>
       <c r="G16" s="16"/>
@@ -5224,10 +5224,10 @@
       <c r="B17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="18"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="15"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -5240,10 +5240,10 @@
     </row>
     <row r="18" spans="2:15" ht="17.25" thickBot="1">
       <c r="B18" s="4"/>
-      <c r="C18" s="18"/>
+      <c r="C18" s="15"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="15"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="28"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
@@ -5258,25 +5258,25 @@
       <c r="B19" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="21"/>
-      <c r="O19" s="22"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="20"/>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="6"/>
-      <c r="C20" s="18"/>
+      <c r="C20" s="15"/>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
@@ -5292,30 +5292,38 @@
     </row>
     <row r="21" spans="2:15" ht="17.25" thickBot="1">
       <c r="B21" s="10"/>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
-      <c r="K21" s="24"/>
-      <c r="L21" s="24"/>
-      <c r="M21" s="24"/>
-      <c r="N21" s="24"/>
-      <c r="O21" s="25"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="F14:O14"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="F18:O18"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="C4:O4"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C3:O3"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="J9:O9"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="F12:O12"/>
     <mergeCell ref="C19:O19"/>
     <mergeCell ref="C20:O20"/>
     <mergeCell ref="C21:O21"/>
@@ -5325,20 +5333,12 @@
     <mergeCell ref="F16:O16"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="F17:O17"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="J9:O9"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:O11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:O12"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="C4:O4"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C3:O3"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="C7:O7"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="F14:O14"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F18:O18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5352,46 +5352,46 @@
   <sheetData>
     <row r="1" spans="2:15" ht="17.25" thickBot="1"/>
     <row r="2" spans="2:15" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="26"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="22"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2"/>
-      <c r="C4" s="18"/>
+      <c r="C4" s="15"/>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -5407,7 +5407,7 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2"/>
-      <c r="C5" s="18"/>
+      <c r="C5" s="15"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -5425,7 +5425,7 @@
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="18"/>
+      <c r="C6" s="15"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -5441,7 +5441,7 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="6"/>
-      <c r="C7" s="18"/>
+      <c r="C7" s="15"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -5459,14 +5459,14 @@
       <c r="B8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="15"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="28"/>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
@@ -5475,14 +5475,14 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="6"/>
-      <c r="C9" s="18"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="15"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="28"/>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
@@ -5493,7 +5493,7 @@
       <c r="B10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="18"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -5509,7 +5509,7 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="6"/>
-      <c r="C11" s="18"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -5527,10 +5527,10 @@
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="18"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="15"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -5543,10 +5543,10 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="6"/>
-      <c r="C13" s="18"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
@@ -5561,10 +5561,10 @@
       <c r="B14" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="18"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -5579,10 +5579,10 @@
       <c r="B15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="18"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="15"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
@@ -5595,10 +5595,10 @@
     </row>
     <row r="16" spans="2:15" ht="17.25" thickBot="1">
       <c r="B16" s="4"/>
-      <c r="C16" s="18"/>
+      <c r="C16" s="15"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="15"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
@@ -5613,25 +5613,25 @@
       <c r="B17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="22"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="20"/>
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="6"/>
-      <c r="C18" s="18"/>
+      <c r="C18" s="15"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
@@ -5647,21 +5647,21 @@
     </row>
     <row r="19" spans="2:15" ht="17.25" thickBot="1">
       <c r="B19" s="10"/>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="24"/>
-      <c r="N19" s="24"/>
-      <c r="O19" s="25"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="23"/>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="14"/>
@@ -5683,15 +5683,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="F13:O13"/>
-    <mergeCell ref="F14:O14"/>
-    <mergeCell ref="F15:O15"/>
-    <mergeCell ref="F16:O16"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C11:O11"/>
-    <mergeCell ref="C5:O5"/>
-    <mergeCell ref="C4:O4"/>
     <mergeCell ref="C17:O17"/>
     <mergeCell ref="C18:O18"/>
     <mergeCell ref="C19:O19"/>
@@ -5708,6 +5699,15 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F12:O12"/>
+    <mergeCell ref="F13:O13"/>
+    <mergeCell ref="F14:O14"/>
+    <mergeCell ref="F15:O15"/>
+    <mergeCell ref="F16:O16"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C5:O5"/>
+    <mergeCell ref="C4:O4"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>